<commit_message>
Adición de casos de formularios Exp y Gto a la creación de los origenes y destino
</commit_message>
<xml_diff>
--- a/resultados/Swift_completos.xlsx
+++ b/resultados/Swift_completos.xlsx
@@ -7904,7 +7904,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>8035</t>
+        </is>
+      </c>
       <c r="L121" t="inlineStr">
         <is>
           <t>artistic-fabric-mills-private-limited-pnbpus3nnyc-4b99a154</t>
@@ -14840,7 +14844,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K233" t="inlineStr"/>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>8132</t>
+        </is>
+      </c>
       <c r="L233" t="inlineStr">
         <is>
           <t>gid-llc-chasus33xxx-fd5d657c</t>
@@ -21546,7 +21554,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K342" t="inlineStr"/>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>10086</t>
+        </is>
+      </c>
       <c r="L342" t="inlineStr">
         <is>
           <t>shaoxing-ada-textile-co-ltd-bofaus3mxxx-fbdbfae5</t>
@@ -24068,7 +24080,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K383" t="inlineStr"/>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>9101</t>
+        </is>
+      </c>
       <c r="L383" t="inlineStr">
         <is>
           <t>ozel-tekstil-insaat-sanayi-ve-ticaret-pnbpus3nnyc-3bec9adb</t>
@@ -25052,7 +25068,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K399" t="inlineStr"/>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>4019</t>
+        </is>
+      </c>
       <c r="L399" t="inlineStr">
         <is>
           <t>prosperity-textile-h-k-ltd-bktrus33xxx-46b27ee9</t>
@@ -25234,7 +25254,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K402" t="inlineStr"/>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>4017</t>
+        </is>
+      </c>
       <c r="L402" t="inlineStr">
         <is>
           <t>raymond-uco-denim-private-limited-chasus33xxx-392a2c18</t>
@@ -25292,7 +25316,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K403" t="inlineStr"/>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>5022</t>
+        </is>
+      </c>
       <c r="L403" t="inlineStr">
         <is>
           <t>raymond-uco-denim-private-limited-chasus33xxx-392a2c18</t>
@@ -25970,7 +25998,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K414" t="inlineStr"/>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>4043</t>
+        </is>
+      </c>
       <c r="L414" t="inlineStr">
         <is>
           <t>kipas-pazarlama-ve-ticaret-as-bktrus33xxx-90661b18</t>
@@ -26028,7 +26060,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K415" t="inlineStr"/>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>5024</t>
+        </is>
+      </c>
       <c r="L415" t="inlineStr"/>
     </row>
     <row r="416">
@@ -28298,7 +28334,11 @@
           <t>Completo</t>
         </is>
       </c>
-      <c r="K452" t="inlineStr"/>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>9075</t>
+        </is>
+      </c>
       <c r="L452" t="inlineStr">
         <is>
           <t>ozel-tekstil-insaat-sanayi-ve-ticaret-pnbpus3nnyc-3bec9adb</t>

</xml_diff>